<commit_message>
feat: add party logos and update voting forms and documentation flow
</commit_message>
<xml_diff>
--- a/all_voting_form_repeat.xlsx
+++ b/all_voting_form_repeat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Desktop\SurveyCTO_Voting_EVM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72482DA-DA44-4351-9D2A-C7B38265024A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC428C6-8D06-47C6-96A7-181458146DA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="555">
   <si>
     <t>type</t>
   </si>
@@ -1614,15 +1614,6 @@
     <t>tmc</t>
   </si>
   <si>
-    <t>TMC (All India Trinamool Congress)</t>
-  </si>
-  <si>
-    <t>टीएमसी (अखिल भारतीय तृणमूल कांग्रेस)</t>
-  </si>
-  <si>
-    <t>tmc.png</t>
-  </si>
-  <si>
     <t>bsp</t>
   </si>
   <si>
@@ -1741,6 +1732,15 @@
   </si>
   <si>
     <t>वर्तमान जीपीएस निर्देशांक कैप्चर करें.</t>
+  </si>
+  <si>
+    <t>SP (Samajwadi Party)</t>
+  </si>
+  <si>
+    <t>एसपी (समाजवादी पार्टी)</t>
+  </si>
+  <si>
+    <t>sp.png</t>
   </si>
 </sst>
 </file>
@@ -2219,7 +2219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2371,6 +2371,7 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2493,16 +2494,16 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFDBE5F1"/>
-          <bgColor rgb="FFDBE5F1"/>
+          <fgColor rgb="FF99BCE7"/>
+          <bgColor rgb="FF99BCE7"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF99BCE7"/>
-          <bgColor rgb="FF99BCE7"/>
+          <fgColor rgb="FFDBE5F1"/>
+          <bgColor rgb="FFDBE5F1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2517,8 +2518,16 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE7D480"/>
-          <bgColor rgb="FFE7D480"/>
+          <fgColor rgb="FFBA005D"/>
+          <bgColor rgb="FFBA005D"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE3E0CF"/>
+          <bgColor rgb="FFE3E0CF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2533,16 +2542,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE3E0CF"/>
-          <bgColor rgb="FFE3E0CF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBA005D"/>
-          <bgColor rgb="FFBA005D"/>
+          <fgColor rgb="FFE7D480"/>
+          <bgColor rgb="FFE7D480"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2557,8 +2558,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFEAF1DD"/>
-          <bgColor rgb="FFEAF1DD"/>
+          <fgColor rgb="FFF2DBDA"/>
+          <bgColor rgb="FFF2DBDA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2573,8 +2574,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF2DBDA"/>
-          <bgColor rgb="FFF2DBDA"/>
+          <fgColor rgb="FFEAF1DD"/>
+          <bgColor rgb="FFEAF1DD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2607,6 +2608,110 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFFF6969"/>
           <bgColor rgb="FFFF6969"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2653,104 +2758,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEEB400"/>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
+          <fgColor rgb="FF99BCE7"/>
+          <bgColor rgb="FF99BCE7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2765,8 +2774,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF99BCE7"/>
-          <bgColor rgb="FF99BCE7"/>
+          <fgColor rgb="FFFBD4B4"/>
+          <bgColor rgb="FFFBD4B4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2781,16 +2790,32 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFBD4B4"/>
-          <bgColor rgb="FFFBD4B4"/>
+          <fgColor rgb="FFBA005D"/>
+          <bgColor rgb="FFBA005D"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFBA005D"/>
-          <bgColor rgb="FFBA005D"/>
+          <fgColor rgb="FFE3E0CF"/>
+          <bgColor rgb="FFE3E0CF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDDE8C6"/>
+          <bgColor rgb="FFDDE8C6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE7D480"/>
+          <bgColor rgb="FFE7D480"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2805,30 +2830,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE7D480"/>
-          <bgColor rgb="FFE7D480"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDDE8C6"/>
-          <bgColor rgb="FFDDE8C6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE3E0CF"/>
-          <bgColor rgb="FFE3E0CF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFFFBB57"/>
           <bgColor rgb="FFFFBB57"/>
         </patternFill>
@@ -2837,16 +2838,16 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFCCC0D9"/>
-          <bgColor rgb="FFCCC0D9"/>
+          <fgColor rgb="FFF2DBDA"/>
+          <bgColor rgb="FFF2DBDA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF2DBDA"/>
-          <bgColor rgb="FFF2DBDA"/>
+          <fgColor rgb="FFCCC0D9"/>
+          <bgColor rgb="FFCCC0D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2885,16 +2886,16 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFF6969"/>
-          <bgColor rgb="FFFF6969"/>
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
+          <fgColor rgb="FFFF6969"/>
+          <bgColor rgb="FFFF6969"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2925,16 +2926,104 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="8"/>
-          <bgColor theme="8"/>
+          <fgColor rgb="FFFF9900"/>
+          <bgColor rgb="FFFF9900"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFBBBB59"/>
-          <bgColor rgb="FFBBBB59"/>
+          <fgColor rgb="FFFABF8F"/>
+          <bgColor rgb="FFFABF8F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4685D2"/>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD6E3BC"/>
+          <bgColor rgb="FFD6E3BC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC4BD97"/>
+          <bgColor rgb="FFC4BD97"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC2D69B"/>
+          <bgColor rgb="FFC2D69B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCC97A"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE4E300"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB2A1C7"/>
+          <bgColor rgb="FFB2A1C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE1AAA9"/>
+          <bgColor rgb="FFE1AAA9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2949,56 +3038,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE1AAA9"/>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB2A1C7"/>
-          <bgColor rgb="FFB2A1C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E300"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDCC97A"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC2D69B"/>
-          <bgColor rgb="FFC2D69B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC4BD97"/>
-          <bgColor rgb="FFC4BD97"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF0000"/>
-          <bgColor rgb="FFFF0000"/>
+          <fgColor rgb="FFBFBFBF"/>
+          <bgColor rgb="FFBFBFBF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3013,56 +3054,16 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF2F2F2"/>
-          <bgColor rgb="FFF2F2F2"/>
+          <fgColor theme="8"/>
+          <bgColor theme="8"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFD6E3BC"/>
-          <bgColor rgb="FFD6E3BC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF4685D2"/>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFABF8F"/>
-          <bgColor rgb="FFFABF8F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF9900"/>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
+          <fgColor rgb="FFBBBB59"/>
+          <bgColor rgb="FFBBBB59"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3277,7 +3278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1000"/>
+  <dimension ref="A1:Z999"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
@@ -3449,126 +3450,135 @@
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s">
+        <v>43</v>
+      </c>
+      <c r="N9" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="N10" t="s">
         <v>44</v>
       </c>
+      <c r="V10" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D11" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="N11" t="s">
         <v>44</v>
       </c>
       <c r="V11" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="N12" t="s">
         <v>44</v>
       </c>
-      <c r="V12" t="s">
-        <v>54</v>
-      </c>
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
-      </c>
-      <c r="N13" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>548</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>65</v>
       </c>
       <c r="B15" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>551</v>
+        <v>68</v>
+      </c>
+      <c r="N15" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B16" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="N16" t="s">
         <v>44</v>
@@ -3576,16 +3586,19 @@
     </row>
     <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C17" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
-        <v>72</v>
+        <v>75</v>
+      </c>
+      <c r="L17" t="s">
+        <v>76</v>
       </c>
       <c r="N17" t="s">
         <v>44</v>
@@ -3593,19 +3606,25 @@
     </row>
     <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C18" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D18" t="s">
-        <v>75</v>
-      </c>
-      <c r="L18" t="s">
-        <v>76</v>
+        <v>80</v>
+      </c>
+      <c r="E18" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" t="s">
+        <v>549</v>
+      </c>
+      <c r="H18" t="s">
+        <v>82</v>
       </c>
       <c r="N18" t="s">
         <v>44</v>
@@ -3613,92 +3632,67 @@
     </row>
     <row r="19" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C19" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D19" t="s">
-        <v>80</v>
-      </c>
-      <c r="E19" t="s">
-        <v>81</v>
-      </c>
-      <c r="F19" t="s">
-        <v>552</v>
-      </c>
-      <c r="H19" t="s">
-        <v>82</v>
-      </c>
-      <c r="N19" t="s">
-        <v>44</v>
+        <v>550</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>85</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
-      </c>
-      <c r="C20" t="s">
-        <v>84</v>
-      </c>
-      <c r="D20" t="s">
-        <v>553</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="B21" t="s">
-        <v>60</v>
+        <v>86</v>
+      </c>
+      <c r="C21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" t="s">
+        <v>547</v>
+      </c>
+      <c r="N21" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D22" t="s">
-        <v>550</v>
+        <v>92</v>
+      </c>
+      <c r="E22" t="s">
+        <v>93</v>
+      </c>
+      <c r="F22" t="s">
+        <v>551</v>
       </c>
       <c r="N22" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>89</v>
-      </c>
-      <c r="B23" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" t="s">
-        <v>91</v>
-      </c>
-      <c r="D23" t="s">
-        <v>92</v>
-      </c>
-      <c r="E23" t="s">
-        <v>93</v>
-      </c>
-      <c r="F23" t="s">
-        <v>554</v>
-      </c>
-      <c r="N23" t="s">
         <v>44</v>
       </c>
     </row>
+    <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="24" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -4675,62 +4669,61 @@
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <conditionalFormatting sqref="A1:W1000 X11:Z15">
-    <cfRule type="expression" dxfId="80" priority="20" stopIfTrue="1">
+  <conditionalFormatting sqref="X10:Z14 A1:W999">
+    <cfRule type="expression" dxfId="80" priority="17" stopIfTrue="1">
+      <formula>$A1="file"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="79" priority="18" stopIfTrue="1">
+      <formula>$A1="enumerator"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="78" priority="19" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1, 14)="sensor_stream ", LEN($A1)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1, 15)))), AND(LEFT($A1, 17)="sensor_statistic ", LEN($A1)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1, 18)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="77" priority="20" stopIfTrue="1">
       <formula>$A1="comments"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="79" priority="34" stopIfTrue="1">
-      <formula>$A1="end repeat"</formula>
+    <cfRule type="expression" dxfId="76" priority="21" stopIfTrue="1">
+      <formula>OR($A1="audio", $A1="video")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="78" priority="33" stopIfTrue="1">
+    <cfRule type="expression" dxfId="75" priority="22" stopIfTrue="1">
+      <formula>$A1="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="74" priority="23" stopIfTrue="1">
+      <formula>OR($A1="date", $A1="datetime", $A1="time")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="73" priority="24" stopIfTrue="1">
+      <formula>OR($A1="calculate", $A1="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="72" priority="25" stopIfTrue="1">
+      <formula>$A1="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="71" priority="26" stopIfTrue="1">
+      <formula>$A1="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="70" priority="27" stopIfTrue="1">
+      <formula>OR($A1="geopoint", $A1="geoshape", $A1="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="69" priority="28" stopIfTrue="1">
+      <formula>OR($A1="audio audit", $A1="text audit", $A1="speed violations count", $A1="speed violations list", $A1="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="68" priority="29" stopIfTrue="1">
+      <formula>OR($A1="username", $A1="phonenumber", $A1="start", $A1="end", $A1="deviceid", $A1="subscriberid", $A1="simserial", $A1="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="67" priority="30" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1, 16)="select_multiple ", LEN($A1)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1, 17)))), AND(LEFT($A1, 11)="select_one ", LEN($A1)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="66" priority="31" stopIfTrue="1">
+      <formula>$A1="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="65" priority="32" stopIfTrue="1">
+      <formula>$A1="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="64" priority="33" stopIfTrue="1">
       <formula>$A1="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="32" stopIfTrue="1">
-      <formula>$A1="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="76" priority="31" stopIfTrue="1">
-      <formula>$A1="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="75" priority="30" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1, 16)="select_multiple ", LEN($A1)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1, 17)))), AND(LEFT($A1, 11)="select_one ", LEN($A1)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="74" priority="29" stopIfTrue="1">
-      <formula>OR($A1="username", $A1="phonenumber", $A1="start", $A1="end", $A1="deviceid", $A1="subscriberid", $A1="simserial", $A1="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="73" priority="19" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1, 14)="sensor_stream ", LEN($A1)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1, 15)))), AND(LEFT($A1, 17)="sensor_statistic ", LEN($A1)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1, 18)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="72" priority="28" stopIfTrue="1">
-      <formula>OR($A1="audio audit", $A1="text audit", $A1="speed violations count", $A1="speed violations list", $A1="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="71" priority="27" stopIfTrue="1">
-      <formula>OR($A1="geopoint", $A1="geoshape", $A1="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="70" priority="26" stopIfTrue="1">
-      <formula>$A1="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="69" priority="25" stopIfTrue="1">
-      <formula>$A1="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="68" priority="24" stopIfTrue="1">
-      <formula>OR($A1="calculate", $A1="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="67" priority="23" stopIfTrue="1">
-      <formula>OR($A1="date", $A1="datetime", $A1="time")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="66" priority="22" stopIfTrue="1">
-      <formula>$A1="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="65" priority="21" stopIfTrue="1">
-      <formula>OR($A1="audio", $A1="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="64" priority="17" stopIfTrue="1">
-      <formula>$A1="file"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="63" priority="18" stopIfTrue="1">
-      <formula>$A1="enumerator"</formula>
+    <cfRule type="expression" dxfId="63" priority="34" stopIfTrue="1">
+      <formula>$A1="end repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="62" priority="35" stopIfTrue="1">
       <formula>$A1="begin repeat"</formula>
@@ -4742,76 +4735,76 @@
       <formula>$A1="begin group"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B1000 F1:F1000">
-    <cfRule type="expression" dxfId="59" priority="39" stopIfTrue="1">
+  <conditionalFormatting sqref="B1:B999 F1:F999">
+    <cfRule type="expression" dxfId="59" priority="8" stopIfTrue="1">
+      <formula>OR($A1="audio audit", $A1="text audit", $A1="speed violations count", $A1="speed violations list", $A1="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="58" priority="39" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1, 14)="sensor_stream ", LEN($A1)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1, 15)))), AND(LEFT($A1, 17)="sensor_statistic ", LEN($A1)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1, 18)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="58" priority="8" stopIfTrue="1">
-      <formula>OR($A1="audio audit", $A1="text audit", $A1="speed violations count", $A1="speed violations list", $A1="speed violations audit")</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B1000 N1:N1000">
+  <conditionalFormatting sqref="B1:B999 N1:N999">
     <cfRule type="expression" dxfId="57" priority="13" stopIfTrue="1">
       <formula>OR($A1="calculate", $A1="calculate_here")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B1000">
+  <conditionalFormatting sqref="B1:B999">
     <cfRule type="expression" dxfId="56" priority="38" stopIfTrue="1">
       <formula>$A1="comments"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:C1000 F1:F1000 I1:I1000">
+  <conditionalFormatting sqref="B1:C999 F1:F999 I1:I999">
     <cfRule type="expression" dxfId="55" priority="1" stopIfTrue="1">
       <formula>$A1="begin group"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:C1000 F1:F1000">
+  <conditionalFormatting sqref="B1:C999 F1:F999">
     <cfRule type="expression" dxfId="54" priority="7" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1, 16)="select_multiple ", LEN($A1)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1, 17)))), AND(LEFT($A1, 11)="select_one ", LEN($A1)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1, 12)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="15" stopIfTrue="1">
+    <cfRule type="expression" dxfId="53" priority="14" stopIfTrue="1">
+      <formula>OR($A1="date", $A1="datetime", $A1="time")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="52" priority="15" stopIfTrue="1">
       <formula>$A1="image"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="14" stopIfTrue="1">
-      <formula>OR($A1="date", $A1="datetime", $A1="time")</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:C1000 I1:I1000 O1:O1000">
+  <conditionalFormatting sqref="B1:C999 I1:I999 O1:O999">
     <cfRule type="expression" dxfId="51" priority="2" stopIfTrue="1">
       <formula>$A1="begin repeat"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:C1000">
-    <cfRule type="expression" dxfId="50" priority="12" stopIfTrue="1">
-      <formula>OR($A1="geopoint", $A1="geoshape", $A1="geotrace")</formula>
+  <conditionalFormatting sqref="B1:C999">
+    <cfRule type="expression" dxfId="50" priority="9" stopIfTrue="1">
+      <formula>$A1="file"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="49" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="49" priority="10" stopIfTrue="1">
+      <formula>$A1="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="11" stopIfTrue="1">
       <formula>$A1="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="10" stopIfTrue="1">
-      <formula>$A1="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="47" priority="9" stopIfTrue="1">
-      <formula>$A1="file"</formula>
+    <cfRule type="expression" dxfId="47" priority="12" stopIfTrue="1">
+      <formula>OR($A1="geopoint", $A1="geoshape", $A1="geotrace")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="46" priority="16" stopIfTrue="1">
       <formula>OR($A1="audio", $A1="video")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:D1000 F1:F1000">
-    <cfRule type="expression" dxfId="45" priority="4" stopIfTrue="1">
+  <conditionalFormatting sqref="B1:D999 F1:F999">
+    <cfRule type="expression" dxfId="45" priority="3" stopIfTrue="1">
+      <formula>$A1="enumerator"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="4" stopIfTrue="1">
       <formula>$A1="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="3" stopIfTrue="1">
-      <formula>$A1="enumerator"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:D999 G1:H999">
+    <cfRule type="expression" dxfId="43" priority="5" stopIfTrue="1">
+      <formula>$A1="integer"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:D1000 G1:H1000">
-    <cfRule type="expression" dxfId="43" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="42" priority="6" stopIfTrue="1">
       <formula>$A1="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="42" priority="5" stopIfTrue="1">
-      <formula>$A1="integer"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.74791666666666667" right="0.74791666666666667" top="0.98402777777777772" bottom="0.98402777777777772" header="0" footer="0"/>
@@ -5418,14 +5411,14 @@
       <c r="B38" t="s">
         <v>511</v>
       </c>
-      <c r="C38" t="s">
-        <v>512</v>
-      </c>
-      <c r="D38" t="s">
-        <v>513</v>
-      </c>
-      <c r="E38" t="s">
-        <v>514</v>
+      <c r="C38" s="61" t="s">
+        <v>552</v>
+      </c>
+      <c r="D38" s="61" t="s">
+        <v>553</v>
+      </c>
+      <c r="E38" s="61" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -5433,16 +5426,16 @@
         <v>498</v>
       </c>
       <c r="B39" t="s">
+        <v>512</v>
+      </c>
+      <c r="C39" t="s">
+        <v>513</v>
+      </c>
+      <c r="D39" t="s">
+        <v>514</v>
+      </c>
+      <c r="E39" t="s">
         <v>515</v>
-      </c>
-      <c r="C39" t="s">
-        <v>516</v>
-      </c>
-      <c r="D39" t="s">
-        <v>517</v>
-      </c>
-      <c r="E39" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -5450,16 +5443,16 @@
         <v>498</v>
       </c>
       <c r="B40" t="s">
+        <v>516</v>
+      </c>
+      <c r="C40" t="s">
+        <v>517</v>
+      </c>
+      <c r="D40" t="s">
+        <v>518</v>
+      </c>
+      <c r="E40" t="s">
         <v>519</v>
-      </c>
-      <c r="C40" t="s">
-        <v>520</v>
-      </c>
-      <c r="D40" t="s">
-        <v>521</v>
-      </c>
-      <c r="E40" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -5467,16 +5460,16 @@
         <v>498</v>
       </c>
       <c r="B41" t="s">
+        <v>520</v>
+      </c>
+      <c r="C41" t="s">
+        <v>521</v>
+      </c>
+      <c r="D41" t="s">
+        <v>522</v>
+      </c>
+      <c r="E41" t="s">
         <v>523</v>
-      </c>
-      <c r="C41" t="s">
-        <v>524</v>
-      </c>
-      <c r="D41" t="s">
-        <v>525</v>
-      </c>
-      <c r="E41" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -5484,13 +5477,13 @@
         <v>423</v>
       </c>
       <c r="B42" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="C42" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="D42" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="F42" t="s">
         <v>414</v>
@@ -5501,13 +5494,13 @@
         <v>423</v>
       </c>
       <c r="B43" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="C43" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="D43" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="F43" t="s">
         <v>417</v>
@@ -5518,13 +5511,13 @@
         <v>423</v>
       </c>
       <c r="B44" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="C44" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="D44" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="F44" t="s">
         <v>420</v>
@@ -5535,16 +5528,16 @@
         <v>442</v>
       </c>
       <c r="B45" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="C45" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="D45" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="F45" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -5552,16 +5545,16 @@
         <v>442</v>
       </c>
       <c r="B46" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="C46" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="D46" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="F46" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -5569,16 +5562,16 @@
         <v>442</v>
       </c>
       <c r="B47" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="C47" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="D47" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="F47" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -5586,16 +5579,16 @@
         <v>442</v>
       </c>
       <c r="B48" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C48" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="D48" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="F48" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -5603,16 +5596,16 @@
         <v>442</v>
       </c>
       <c r="B49" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="C49" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="D49" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="F49" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -5620,16 +5613,16 @@
         <v>442</v>
       </c>
       <c r="B50" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="C50" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="D50" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="F50" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
     </row>
   </sheetData>
@@ -5693,14 +5686,14 @@
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="C2" s="5" t="str">
         <f ca="1">TEXT(YEAR(NOW())-2000, "00") &amp; TEXT(MONTH(NOW()), "00") &amp; TEXT(DAY(NOW()), "00") &amp; TEXT(HOUR(NOW()), "00") &amp; TEXT(MINUTE(NOW()), "00")</f>
-        <v>2607082137</v>
+        <v>2607082151</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -5724,10 +5717,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="71" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="71"/>
+      <c r="B1" s="72"/>
       <c r="C1" s="11"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -5759,8 +5752,8 @@
       <c r="AE1" s="2"/>
     </row>
     <row r="2" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="63"/>
-      <c r="B2" s="64"/>
+      <c r="A2" s="64"/>
+      <c r="B2" s="65"/>
       <c r="C2" s="11"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -5792,10 +5785,10 @@
       <c r="AE2" s="2"/>
     </row>
     <row r="3" spans="1:31" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="72" t="s">
+      <c r="A3" s="73" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="64"/>
+      <c r="B3" s="65"/>
       <c r="C3" s="11"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -5827,10 +5820,10 @@
       <c r="AE3" s="2"/>
     </row>
     <row r="4" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="61" t="s">
+      <c r="A4" s="62" t="s">
         <v>103</v>
       </c>
-      <c r="B4" s="62"/>
+      <c r="B4" s="63"/>
       <c r="C4" s="11"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -6193,10 +6186,10 @@
       <c r="AE9" s="2"/>
     </row>
     <row r="10" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="65" t="s">
+      <c r="A10" s="66" t="s">
         <v>156</v>
       </c>
-      <c r="B10" s="66"/>
+      <c r="B10" s="67"/>
       <c r="C10" s="23"/>
       <c r="D10" s="24"/>
       <c r="E10" s="24"/>
@@ -9334,10 +9327,10 @@
       <c r="C90" s="11"/>
     </row>
     <row r="91" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="73" t="s">
+      <c r="A91" s="74" t="s">
         <v>273</v>
       </c>
-      <c r="B91" s="69"/>
+      <c r="B91" s="70"/>
       <c r="C91" s="32"/>
       <c r="D91" s="33"/>
       <c r="E91" s="2"/>
@@ -9369,11 +9362,11 @@
       <c r="AE91" s="2"/>
     </row>
     <row r="92" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="67" t="s">
+      <c r="A92" s="68" t="s">
         <v>274</v>
       </c>
-      <c r="B92" s="68"/>
-      <c r="C92" s="69"/>
+      <c r="B92" s="69"/>
+      <c r="C92" s="70"/>
       <c r="D92" s="33"/>
       <c r="E92" s="2"/>
       <c r="F92" s="2"/>
@@ -12616,59 +12609,59 @@
     <mergeCell ref="A91:B91"/>
   </mergeCells>
   <conditionalFormatting sqref="A6:AD6">
-    <cfRule type="expression" dxfId="41" priority="25" stopIfTrue="1">
+    <cfRule type="expression" dxfId="41" priority="15" stopIfTrue="1">
+      <formula>$A6="comments"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="40" priority="16" stopIfTrue="1">
+      <formula>OR($A6="audio", $A6="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="39" priority="17" stopIfTrue="1">
+      <formula>$A6="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="38" priority="18" stopIfTrue="1">
+      <formula>OR($A6="date", $A6="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="37" priority="19" stopIfTrue="1">
+      <formula>OR($A6="calculate", $A6="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="36" priority="20" stopIfTrue="1">
+      <formula>$A6="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="35" priority="21" stopIfTrue="1">
+      <formula>$A6="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="34" priority="22" stopIfTrue="1">
+      <formula>$A6="geopoint"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="33" priority="23" stopIfTrue="1">
+      <formula>OR($A6="audio audit", $A6="text audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="32" priority="24" stopIfTrue="1">
+      <formula>OR($A6="phonenumber", $A6="start", $A6="end", $A6="deviceid", $A6="subscriberid", $A6="simserial")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="31" priority="25" stopIfTrue="1">
       <formula>OR(AND(LEFT($A6, 16)="select_multiple ", LEN($A6)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A6, 17)))), AND(LEFT($A6, 11)="select_one ", LEN($A6)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A6, 12)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="20" stopIfTrue="1">
-      <formula>$A6="note"</formula>
+    <cfRule type="expression" dxfId="30" priority="26" stopIfTrue="1">
+      <formula>$A6="decimal"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="21" stopIfTrue="1">
-      <formula>$A6="barcode"</formula>
+    <cfRule type="expression" dxfId="29" priority="27" stopIfTrue="1">
+      <formula>$A6="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="32" stopIfTrue="1">
-      <formula>$A6="begin group"</formula>
+    <cfRule type="expression" dxfId="28" priority="28" stopIfTrue="1">
+      <formula>$A6="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="31" stopIfTrue="1">
+    <cfRule type="expression" dxfId="27" priority="29" stopIfTrue="1">
+      <formula>$A6="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="30" stopIfTrue="1">
+      <formula>$A6="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="25" priority="31" stopIfTrue="1">
       <formula>$A6="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="22" stopIfTrue="1">
-      <formula>$A6="geopoint"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="35" priority="30" stopIfTrue="1">
-      <formula>$A6="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="34" priority="29" stopIfTrue="1">
-      <formula>$A6="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="33" priority="28" stopIfTrue="1">
-      <formula>$A6="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="32" priority="27" stopIfTrue="1">
-      <formula>$A6="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="31" priority="26" stopIfTrue="1">
-      <formula>$A6="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="30" priority="24" stopIfTrue="1">
-      <formula>OR($A6="phonenumber", $A6="start", $A6="end", $A6="deviceid", $A6="subscriberid", $A6="simserial")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="29" priority="23" stopIfTrue="1">
-      <formula>OR($A6="audio audit", $A6="text audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="28" priority="15" stopIfTrue="1">
-      <formula>$A6="comments"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="27" priority="16" stopIfTrue="1">
-      <formula>OR($A6="audio", $A6="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="26" priority="17" stopIfTrue="1">
-      <formula>$A6="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="25" priority="18" stopIfTrue="1">
-      <formula>OR($A6="date", $A6="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="19" stopIfTrue="1">
-      <formula>OR($A6="calculate", $A6="calculate_here")</formula>
+    <cfRule type="expression" dxfId="24" priority="32" stopIfTrue="1">
+      <formula>$A6="begin group"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6 H6">
@@ -12692,14 +12685,14 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6 H6">
-    <cfRule type="expression" dxfId="19" priority="13" stopIfTrue="1">
-      <formula>$A6="image"</formula>
+    <cfRule type="expression" dxfId="19" priority="6" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A6, 16)="select_multiple ", LEN($A6)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A6, 17)))), AND(LEFT($A6, 11)="select_one ", LEN($A6)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A6, 12)))))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="18" priority="12" stopIfTrue="1">
       <formula>OR($A6="date", $A6="datetime")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="6" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A6, 16)="select_multiple ", LEN($A6)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A6, 17)))), AND(LEFT($A6, 11)="select_one ", LEN($A6)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A6, 12)))))</formula>
+    <cfRule type="expression" dxfId="17" priority="13" stopIfTrue="1">
+      <formula>$A6="image"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6 L6 S6">
@@ -12708,17 +12701,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="expression" dxfId="15" priority="14" stopIfTrue="1">
-      <formula>OR($A6="audio", $A6="video")</formula>
+    <cfRule type="expression" dxfId="15" priority="8" stopIfTrue="1">
+      <formula>$A6="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="9" stopIfTrue="1">
+      <formula>$A6="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="10" stopIfTrue="1">
       <formula>$A6="geopoint"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="9" stopIfTrue="1">
-      <formula>$A6="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="8" stopIfTrue="1">
-      <formula>$A6="note"</formula>
+    <cfRule type="expression" dxfId="12" priority="14" stopIfTrue="1">
+      <formula>OR($A6="audio", $A6="video")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:F6 H6">
@@ -12727,11 +12720,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:F6 I6:K6">
-    <cfRule type="expression" dxfId="10" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="4" stopIfTrue="1">
+      <formula>$A6="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="5" stopIfTrue="1">
       <formula>$A6="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="4" stopIfTrue="1">
-      <formula>$A6="integer"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6">
@@ -12832,10 +12825,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="71" t="s">
         <v>383</v>
       </c>
-      <c r="B1" s="71"/>
+      <c r="B1" s="72"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -12890,10 +12883,10 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" spans="1:26" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="72" t="s">
+      <c r="A3" s="73" t="s">
         <v>384</v>
       </c>
-      <c r="B3" s="64"/>
+      <c r="B3" s="65"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -12920,10 +12913,10 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="74" t="s">
+      <c r="A4" s="75" t="s">
         <v>385</v>
       </c>
-      <c r="B4" s="64"/>
+      <c r="B4" s="65"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -12950,10 +12943,10 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="75" t="s">
         <v>386</v>
       </c>
-      <c r="B5" s="64"/>
+      <c r="B5" s="65"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -12980,10 +12973,10 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="62" t="s">
         <v>387</v>
       </c>
-      <c r="B6" s="62"/>
+      <c r="B6" s="63"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -14173,10 +14166,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="80" t="s">
         <v>398</v>
       </c>
-      <c r="B1" s="80"/>
+      <c r="B1" s="81"/>
       <c r="C1" s="54"/>
       <c r="D1" s="54"/>
       <c r="E1" s="54"/>
@@ -14203,8 +14196,8 @@
       <c r="Z1" s="2"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="77"/>
-      <c r="B2" s="78"/>
+      <c r="A2" s="78"/>
+      <c r="B2" s="79"/>
       <c r="C2" s="54"/>
       <c r="D2" s="54"/>
       <c r="E2" s="54"/>
@@ -14231,10 +14224,10 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" spans="1:26" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="76" t="s">
         <v>399</v>
       </c>
-      <c r="B3" s="76"/>
+      <c r="B3" s="77"/>
       <c r="C3" s="54"/>
       <c r="D3" s="54"/>
       <c r="E3" s="54"/>

</xml_diff>